<commit_message>
Add: Fiche évaluation et remise finale
</commit_message>
<xml_diff>
--- a/eval/C64 - Fiche autoévaluation - Partie 2.xlsx
+++ b/eval/C64 - Fiche autoévaluation - Partie 2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Google Drive\Professionnel\ETS\Enseignement\GPA434\2018_3_automne\Laboratoires\Laboratoire 3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\1379670\Desktop\Robot5\eval\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41319B72-8DCD-4E89-B88B-C986378D3009}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1097CE1E-C72F-45B8-B64E-72BECACFFC04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Évaluation" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,12 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -33,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="102">
   <si>
     <t>Étudiant 1</t>
   </si>
@@ -321,6 +326,24 @@
   </si>
   <si>
     <t>débrouillardise, initiative, amène des solutions pertinentes et de haut niveau, motivation d'équipe …</t>
+  </si>
+  <si>
+    <t>Dumesnil Laurent</t>
+  </si>
+  <si>
+    <t>Proulx Jérémie</t>
+  </si>
+  <si>
+    <t>Julien Lamontagne</t>
+  </si>
+  <si>
+    <t>Yanis Boumazouzi</t>
+  </si>
+  <si>
+    <t>Isabela Forest Martinez</t>
+  </si>
+  <si>
+    <t>Marie Joëlle Isabelle Ndioukane</t>
   </si>
 </sst>
 </file>
@@ -1341,93 +1364,6 @@
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="5" borderId="42" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="5" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="38" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="39" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" textRotation="90" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
@@ -1471,49 +1407,17 @@
       <alignment horizontal="right"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="42" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="36" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
       <protection hidden="1"/>
@@ -1528,7 +1432,126 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="38" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="39" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" textRotation="90" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="36" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="42" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="42" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="43" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="42" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
@@ -1543,19 +1566,9 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
+    <cellStyle name="Pourcentage" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="4">
-    <dxf>
-      <font>
-        <color theme="0" tint="-4.9989318521683403E-2"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF800000"/>
@@ -1564,15 +1577,6 @@
         <bottom style="thin">
           <color rgb="FF800000"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF800000"/>
-      </font>
-      <border>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -1594,6 +1598,25 @@
           <color rgb="FF800000"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF800000"/>
+      </font>
+      <border>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1620,9 +1643,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1660,7 +1683,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1766,7 +1789,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1908,7 +1931,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1917,20 +1940,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:AA80"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3" style="49" customWidth="1"/>
     <col min="2" max="2" width="7" style="49" customWidth="1"/>
     <col min="3" max="3" width="3" style="49" customWidth="1"/>
     <col min="4" max="4" width="12" style="49" customWidth="1"/>
-    <col min="5" max="5" width="18.86328125" style="49" customWidth="1"/>
-    <col min="6" max="6" width="34.46484375" style="49" customWidth="1"/>
-    <col min="7" max="9" width="13.73046875" style="2" customWidth="1"/>
-    <col min="10" max="10" width="6.73046875" style="2" customWidth="1"/>
-    <col min="11" max="11" width="13.73046875" style="2" customWidth="1"/>
-    <col min="12" max="12" width="11.265625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="12.3984375" style="3" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="11.265625" style="2" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="18.81640625" style="49" customWidth="1"/>
+    <col min="6" max="6" width="34.453125" style="49" customWidth="1"/>
+    <col min="7" max="9" width="13.7265625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="6.7265625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="13.7265625" style="2" customWidth="1"/>
+    <col min="12" max="12" width="11.26953125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="12.36328125" style="3" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="11.26953125" style="2" hidden="1" customWidth="1"/>
     <col min="15" max="22" width="9" style="2" hidden="1" customWidth="1"/>
     <col min="23" max="23" width="10" style="2" hidden="1" customWidth="1"/>
     <col min="24" max="25" width="9" style="49" hidden="1" customWidth="1"/>
@@ -1938,148 +1961,148 @@
     <col min="28" max="16384" width="9" style="49"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="77" t="s">
+    <row r="2" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="89" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="77"/>
-      <c r="D3" s="69" t="s">
+    <row r="3" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="89"/>
+      <c r="D3" s="109" t="s">
         <v>53</v>
       </c>
-      <c r="E3" s="70"/>
-      <c r="F3" s="70"/>
-      <c r="G3" s="71">
-        <v>4</v>
-      </c>
-      <c r="H3" s="71"/>
-      <c r="I3" s="71"/>
-      <c r="J3" s="71"/>
-      <c r="K3" s="72"/>
-    </row>
-    <row r="4" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B4" s="77"/>
-    </row>
-    <row r="5" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B5" s="77"/>
-      <c r="D5" s="69" t="s">
+      <c r="E3" s="110"/>
+      <c r="F3" s="110"/>
+      <c r="G3" s="111">
+        <v>6</v>
+      </c>
+      <c r="H3" s="111"/>
+      <c r="I3" s="111"/>
+      <c r="J3" s="111"/>
+      <c r="K3" s="112"/>
+    </row>
+    <row r="4" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="89"/>
+    </row>
+    <row r="5" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="89"/>
+      <c r="D5" s="109" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="70"/>
-      <c r="F5" s="70"/>
-      <c r="G5" s="102">
+      <c r="E5" s="110"/>
+      <c r="F5" s="110"/>
+      <c r="G5" s="93">
         <v>0.85</v>
       </c>
-      <c r="H5" s="102"/>
-      <c r="I5" s="102"/>
-      <c r="J5" s="102"/>
-      <c r="K5" s="103"/>
-    </row>
-    <row r="6" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B6" s="77"/>
-      <c r="G6" s="79" t="s">
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="93"/>
+      <c r="K5" s="94"/>
+    </row>
+    <row r="6" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B6" s="89"/>
+      <c r="G6" s="95" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="79"/>
-      <c r="I6" s="79"/>
-      <c r="J6" s="79"/>
-      <c r="K6" s="79"/>
-    </row>
-    <row r="7" spans="2:22" x14ac:dyDescent="0.45">
-      <c r="B7" s="77"/>
-      <c r="D7" s="89" t="s">
+      <c r="H6" s="95"/>
+      <c r="I6" s="95"/>
+      <c r="J6" s="95"/>
+      <c r="K6" s="95"/>
+    </row>
+    <row r="7" spans="2:22" x14ac:dyDescent="0.35">
+      <c r="B7" s="89"/>
+      <c r="D7" s="107" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="90"/>
-      <c r="F7" s="90"/>
-      <c r="G7" s="104">
+      <c r="E7" s="108"/>
+      <c r="F7" s="108"/>
+      <c r="G7" s="96">
         <v>0.6</v>
       </c>
-      <c r="H7" s="104"/>
-      <c r="I7" s="104"/>
-      <c r="J7" s="104"/>
-      <c r="K7" s="105"/>
-    </row>
-    <row r="8" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B8" s="77"/>
-      <c r="D8" s="87" t="s">
+      <c r="H7" s="96"/>
+      <c r="I7" s="96"/>
+      <c r="J7" s="96"/>
+      <c r="K7" s="97"/>
+    </row>
+    <row r="8" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B8" s="89"/>
+      <c r="D8" s="105" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="80">
+      <c r="E8" s="106"/>
+      <c r="F8" s="106"/>
+      <c r="G8" s="98">
         <f>1-G7</f>
         <v>0.4</v>
       </c>
-      <c r="H8" s="80"/>
-      <c r="I8" s="80"/>
-      <c r="J8" s="80"/>
-      <c r="K8" s="81"/>
+      <c r="H8" s="98"/>
+      <c r="I8" s="98"/>
+      <c r="J8" s="98"/>
+      <c r="K8" s="99"/>
       <c r="V8" s="4"/>
     </row>
-    <row r="9" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B9" s="77"/>
+    <row r="9" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B9" s="89"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
-      <c r="G9" s="82"/>
-      <c r="H9" s="82"/>
-      <c r="I9" s="82"/>
-      <c r="J9" s="82"/>
-      <c r="K9" s="82"/>
-    </row>
-    <row r="10" spans="2:22" x14ac:dyDescent="0.45">
-      <c r="B10" s="77"/>
-      <c r="D10" s="85" t="s">
+      <c r="G9" s="100"/>
+      <c r="H9" s="100"/>
+      <c r="I9" s="100"/>
+      <c r="J9" s="100"/>
+      <c r="K9" s="100"/>
+    </row>
+    <row r="10" spans="2:22" x14ac:dyDescent="0.35">
+      <c r="B10" s="89"/>
+      <c r="D10" s="103" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="86"/>
-      <c r="F10" s="86"/>
-      <c r="G10" s="106">
+      <c r="E10" s="104"/>
+      <c r="F10" s="104"/>
+      <c r="G10" s="91">
         <v>0.5</v>
       </c>
-      <c r="H10" s="106"/>
-      <c r="I10" s="106"/>
-      <c r="J10" s="106"/>
-      <c r="K10" s="107"/>
-    </row>
-    <row r="11" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B11" s="77"/>
-      <c r="D11" s="83" t="s">
+      <c r="H10" s="91"/>
+      <c r="I10" s="91"/>
+      <c r="J10" s="91"/>
+      <c r="K10" s="92"/>
+    </row>
+    <row r="11" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B11" s="89"/>
+      <c r="D11" s="101" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="84"/>
-      <c r="F11" s="84"/>
-      <c r="G11" s="75">
+      <c r="E11" s="102"/>
+      <c r="F11" s="102"/>
+      <c r="G11" s="87">
         <f ca="1">V44</f>
         <v>0</v>
       </c>
-      <c r="H11" s="75"/>
-      <c r="I11" s="75"/>
-      <c r="J11" s="75"/>
-      <c r="K11" s="76"/>
-    </row>
-    <row r="12" spans="2:22" x14ac:dyDescent="0.45">
-      <c r="B12" s="77"/>
+      <c r="H11" s="87"/>
+      <c r="I11" s="87"/>
+      <c r="J11" s="87"/>
+      <c r="K11" s="88"/>
+    </row>
+    <row r="12" spans="2:22" x14ac:dyDescent="0.35">
+      <c r="B12" s="89"/>
       <c r="D12" s="1"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
-      <c r="K12" s="101" t="s">
+      <c r="K12" s="79" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="13" spans="2:22" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:22" x14ac:dyDescent="0.35">
       <c r="D13" s="1"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
     </row>
-    <row r="14" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B14" s="78" t="s">
+    <row r="14" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B14" s="90" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="2:22" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="78"/>
+    <row r="15" spans="2:22" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="90"/>
       <c r="D15" s="21"/>
       <c r="E15" s="22"/>
       <c r="F15" s="22"/>
@@ -2092,32 +2115,32 @@
       <c r="I15" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="J15" s="73" t="s">
+      <c r="J15" s="113" t="s">
         <v>9</v>
       </c>
-      <c r="K15" s="74"/>
-    </row>
-    <row r="16" spans="2:22" x14ac:dyDescent="0.45">
-      <c r="B16" s="78"/>
+      <c r="K15" s="114"/>
+    </row>
+    <row r="16" spans="2:22" x14ac:dyDescent="0.35">
+      <c r="B16" s="90"/>
       <c r="D16" s="12"/>
       <c r="E16" s="13"/>
       <c r="F16" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="G16" s="108">
+      <c r="G16" s="80">
         <v>0.4</v>
       </c>
-      <c r="H16" s="109">
+      <c r="H16" s="81">
         <v>0.4</v>
       </c>
-      <c r="I16" s="110">
+      <c r="I16" s="82">
         <v>0.2</v>
       </c>
       <c r="J16" s="62"/>
       <c r="K16" s="14"/>
     </row>
-    <row r="17" spans="2:27" x14ac:dyDescent="0.45">
-      <c r="B17" s="78"/>
+    <row r="17" spans="2:27" x14ac:dyDescent="0.35">
+      <c r="B17" s="90"/>
       <c r="D17" s="12"/>
       <c r="E17" s="13"/>
       <c r="F17" s="51" t="s">
@@ -2135,8 +2158,8 @@
       <c r="J17" s="9"/>
       <c r="K17" s="14"/>
     </row>
-    <row r="18" spans="2:27" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B18" s="78"/>
+    <row r="18" spans="2:27" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B18" s="90"/>
       <c r="D18" s="12"/>
       <c r="E18" s="53" t="s">
         <v>51</v>
@@ -2150,24 +2173,31 @@
       <c r="J18" s="9"/>
       <c r="K18" s="14"/>
     </row>
-    <row r="19" spans="2:27" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="B19" s="78"/>
+    <row r="19" spans="2:27" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="90"/>
       <c r="C19" s="58">
         <v>1</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="E19" s="63"/>
-      <c r="F19" s="64"/>
+      <c r="E19" s="63">
+        <v>1379670</v>
+      </c>
+      <c r="F19" s="64" t="s">
+        <v>96</v>
+      </c>
       <c r="G19" s="28">
-        <v>0.25</v>
+        <f>(100/6)/100</f>
+        <v>0.16666666666666669</v>
       </c>
       <c r="H19" s="7">
-        <v>0.05</v>
+        <f t="shared" ref="H19:I19" si="0">(100/6)/100</f>
+        <v>0.16666666666666669</v>
       </c>
       <c r="I19" s="29">
-        <v>0.5</v>
+        <f t="shared" si="0"/>
+        <v>0.16666666666666669</v>
       </c>
       <c r="J19" s="60" t="str">
         <f ca="1">IF(V19&gt;0,"- "&amp;TEXT(V19*100,"0.0")&amp;"%",IF(Z19&gt;0,"+ "&amp;TEXT(Z19*100,"0.0")&amp;"%",""))</f>
@@ -2175,24 +2205,24 @@
       </c>
       <c r="K19" s="16">
         <f ca="1">AA19</f>
-        <v>0.80920000000000014</v>
+        <v>0.85000000000000009</v>
       </c>
       <c r="L19" s="34"/>
       <c r="M19" s="46">
-        <f>E19</f>
-        <v>0</v>
+        <f t="shared" ref="M19:M43" si="1">E19</f>
+        <v>1379670</v>
       </c>
       <c r="N19" s="50">
         <f t="array" ref="N19">SUM(G19:I19/$G$17:$I$17*$G$16:$I$16)</f>
-        <v>0.22000000000000003</v>
+        <v>0.16666666666666669</v>
       </c>
       <c r="O19" s="50">
         <f>1/$M$49</f>
-        <v>0.25</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P19" s="4">
         <f>N19/O19</f>
-        <v>0.88000000000000012</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="Q19" s="4">
         <f>$G$5</f>
@@ -2204,15 +2234,15 @@
       </c>
       <c r="S19" s="4">
         <f>P19*Q19*$G$8</f>
-        <v>0.29920000000000008</v>
+        <v>0.34000000000000008</v>
       </c>
       <c r="T19" s="4">
         <f>SUM(R19:S19)</f>
-        <v>0.80920000000000014</v>
+        <v>0.85000000000000009</v>
       </c>
       <c r="U19" s="4">
         <f>MIN(1,T19)</f>
-        <v>0.80920000000000014</v>
+        <v>0.85000000000000009</v>
       </c>
       <c r="V19" s="4">
         <f>T19-U19</f>
@@ -2220,11 +2250,11 @@
       </c>
       <c r="W19" s="4">
         <f>1-U19</f>
-        <v>0.19079999999999986</v>
+        <v>0.14999999999999991</v>
       </c>
       <c r="X19" s="4">
         <f ca="1">W19/$W$44</f>
-        <v>0.31799999999999995</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="Y19" s="4">
         <f ca="1">X19*$V$44</f>
@@ -2236,52 +2266,59 @@
       </c>
       <c r="AA19" s="4">
         <f ca="1">U19+Z19</f>
-        <v>0.80920000000000014</v>
-      </c>
-    </row>
-    <row r="20" spans="2:27" x14ac:dyDescent="0.45">
-      <c r="B20" s="78"/>
+        <v>0.85000000000000009</v>
+      </c>
+    </row>
+    <row r="20" spans="2:27" x14ac:dyDescent="0.35">
+      <c r="B20" s="90"/>
       <c r="C20" s="58">
         <v>2</v>
       </c>
       <c r="D20" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="E20" s="65"/>
-      <c r="F20" s="66"/>
+      <c r="E20" s="65">
+        <v>1746047</v>
+      </c>
+      <c r="F20" s="66" t="s">
+        <v>97</v>
+      </c>
       <c r="G20" s="30">
-        <v>0.25</v>
+        <f t="shared" ref="G20:I24" si="2">(100/6)/100</f>
+        <v>0.16666666666666669</v>
       </c>
       <c r="H20" s="8">
-        <v>0.35</v>
+        <f t="shared" si="2"/>
+        <v>0.16666666666666669</v>
       </c>
       <c r="I20" s="31">
-        <v>0.2</v>
+        <f t="shared" si="2"/>
+        <v>0.16666666666666669</v>
       </c>
       <c r="J20" s="61" t="str">
-        <f t="shared" ref="J20:J43" ca="1" si="0">IF(V20&gt;0,"- "&amp;TEXT(V20*100,"0.0")&amp;"%",IF(Z20&gt;0,"+ "&amp;TEXT(Z20*100,"0.0")&amp;"%",""))</f>
+        <f t="shared" ref="J20:J43" ca="1" si="3">IF(V20&gt;0,"- "&amp;TEXT(V20*100,"0.0")&amp;"%",IF(Z20&gt;0,"+ "&amp;TEXT(Z20*100,"0.0")&amp;"%",""))</f>
         <v/>
       </c>
       <c r="K20" s="18">
-        <f t="shared" ref="K20:K43" ca="1" si="1">AA20</f>
-        <v>0.89080000000000004</v>
+        <f t="shared" ref="K20:K43" ca="1" si="4">AA20</f>
+        <v>0.85000000000000009</v>
       </c>
       <c r="L20" s="34"/>
       <c r="M20" s="46">
-        <f>E20</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>1746047</v>
       </c>
       <c r="N20" s="50">
         <f t="array" ref="N20">SUM(G20:I20/$G$17:$I$17*$G$16:$I$16)</f>
-        <v>0.28000000000000003</v>
+        <v>0.16666666666666669</v>
       </c>
       <c r="O20" s="50">
         <f>1/$M$49</f>
-        <v>0.25</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P20" s="4">
         <f>N20/O20</f>
-        <v>1.1200000000000001</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="Q20" s="4">
         <f>$G$5</f>
@@ -2293,84 +2330,91 @@
       </c>
       <c r="S20" s="4">
         <f>P20*Q20*$G$8</f>
-        <v>0.38080000000000003</v>
+        <v>0.34000000000000008</v>
       </c>
       <c r="T20" s="4">
-        <f t="shared" ref="T20:T22" si="2">SUM(R20:S20)</f>
-        <v>0.89080000000000004</v>
+        <f t="shared" ref="T20:T22" si="5">SUM(R20:S20)</f>
+        <v>0.85000000000000009</v>
       </c>
       <c r="U20" s="4">
         <f>MIN(1,T20)</f>
-        <v>0.89080000000000004</v>
+        <v>0.85000000000000009</v>
       </c>
       <c r="V20" s="4">
-        <f t="shared" ref="V20:V22" si="3">T20-U20</f>
+        <f t="shared" ref="V20:V22" si="6">T20-U20</f>
         <v>0</v>
       </c>
       <c r="W20" s="4">
         <f>1-U20</f>
-        <v>0.10919999999999996</v>
+        <v>0.14999999999999991</v>
       </c>
       <c r="X20" s="4">
         <f ca="1">W20/$W$44</f>
-        <v>0.18200000000000005</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="Y20" s="4">
         <f ca="1">X20*$V$44</f>
         <v>0</v>
       </c>
       <c r="Z20" s="4">
-        <f t="shared" ref="Z20:Z22" ca="1" si="4">Y20*$G$10</f>
+        <f t="shared" ref="Z20:Z22" ca="1" si="7">Y20*$G$10</f>
         <v>0</v>
       </c>
       <c r="AA20" s="4">
         <f ca="1">U20+Z20</f>
-        <v>0.89080000000000004</v>
-      </c>
-    </row>
-    <row r="21" spans="2:27" x14ac:dyDescent="0.45">
-      <c r="B21" s="78"/>
+        <v>0.85000000000000009</v>
+      </c>
+    </row>
+    <row r="21" spans="2:27" x14ac:dyDescent="0.35">
+      <c r="B21" s="90"/>
       <c r="C21" s="58">
         <v>3</v>
       </c>
       <c r="D21" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="E21" s="65"/>
-      <c r="F21" s="66"/>
+      <c r="E21" s="65">
+        <v>869558</v>
+      </c>
+      <c r="F21" s="66" t="s">
+        <v>98</v>
+      </c>
       <c r="G21" s="30">
-        <v>0.25</v>
+        <f t="shared" si="2"/>
+        <v>0.16666666666666669</v>
       </c>
       <c r="H21" s="8">
-        <v>0.3</v>
+        <f t="shared" si="2"/>
+        <v>0.16666666666666669</v>
       </c>
       <c r="I21" s="31">
-        <v>0.15</v>
+        <f t="shared" si="2"/>
+        <v>0.16666666666666669</v>
       </c>
       <c r="J21" s="61" t="str">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
       <c r="K21" s="18">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="4"/>
         <v>0.85000000000000009</v>
       </c>
       <c r="L21" s="34"/>
       <c r="M21" s="46">
-        <f>E21</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>869558</v>
       </c>
       <c r="N21" s="50">
         <f t="array" ref="N21">SUM(G21:I21/$G$17:$I$17*$G$16:$I$16)</f>
-        <v>0.25</v>
+        <v>0.16666666666666669</v>
       </c>
       <c r="O21" s="50">
         <f>1/$M$49</f>
-        <v>0.25</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P21" s="4">
         <f>N21/O21</f>
-        <v>1</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="Q21" s="4">
         <f>$G$5</f>
@@ -2382,10 +2426,10 @@
       </c>
       <c r="S21" s="4">
         <f>P21*Q21*$G$8</f>
-        <v>0.34</v>
+        <v>0.34000000000000008</v>
       </c>
       <c r="T21" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.85000000000000009</v>
       </c>
       <c r="U21" s="4">
@@ -2393,7 +2437,7 @@
         <v>0.85000000000000009</v>
       </c>
       <c r="V21" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="W21" s="4">
@@ -2402,14 +2446,14 @@
       </c>
       <c r="X21" s="4">
         <f ca="1">W21/$W$44</f>
-        <v>0.25</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="Y21" s="4">
         <f ca="1">X21*$V$44</f>
         <v>0</v>
       </c>
       <c r="Z21" s="4">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="7"/>
         <v>0</v>
       </c>
       <c r="AA21" s="4">
@@ -2417,49 +2461,56 @@
         <v>0.85000000000000009</v>
       </c>
     </row>
-    <row r="22" spans="2:27" x14ac:dyDescent="0.45">
-      <c r="B22" s="78"/>
+    <row r="22" spans="2:27" x14ac:dyDescent="0.35">
+      <c r="B22" s="90"/>
       <c r="C22" s="58">
         <v>4</v>
       </c>
       <c r="D22" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E22" s="65"/>
-      <c r="F22" s="66"/>
+      <c r="E22" s="65">
+        <v>2290619</v>
+      </c>
+      <c r="F22" s="66" t="s">
+        <v>99</v>
+      </c>
       <c r="G22" s="30">
-        <v>0.25</v>
+        <f t="shared" si="2"/>
+        <v>0.16666666666666669</v>
       </c>
       <c r="H22" s="8">
-        <v>0.3</v>
+        <f t="shared" si="2"/>
+        <v>0.16666666666666669</v>
       </c>
       <c r="I22" s="31">
-        <v>0.15</v>
+        <f t="shared" si="2"/>
+        <v>0.16666666666666669</v>
       </c>
       <c r="J22" s="61" t="str">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
       <c r="K22" s="18">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="4"/>
         <v>0.85000000000000009</v>
       </c>
       <c r="L22" s="34"/>
       <c r="M22" s="46">
-        <f>E22</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>2290619</v>
       </c>
       <c r="N22" s="50">
         <f t="array" ref="N22">SUM(G22:I22/$G$17:$I$17*$G$16:$I$16)</f>
-        <v>0.25</v>
+        <v>0.16666666666666669</v>
       </c>
       <c r="O22" s="50">
         <f>1/$M$49</f>
-        <v>0.25</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P22" s="4">
         <f>N22/O22</f>
-        <v>1</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="Q22" s="4">
         <f>$G$5</f>
@@ -2471,10 +2522,10 @@
       </c>
       <c r="S22" s="4">
         <f>P22*Q22*$G$8</f>
-        <v>0.34</v>
+        <v>0.34000000000000008</v>
       </c>
       <c r="T22" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.85000000000000009</v>
       </c>
       <c r="U22" s="4">
@@ -2482,7 +2533,7 @@
         <v>0.85000000000000009</v>
       </c>
       <c r="V22" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="W22" s="4">
@@ -2491,14 +2542,14 @@
       </c>
       <c r="X22" s="4">
         <f ca="1">W22/$W$44</f>
-        <v>0.25</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="Y22" s="4">
         <f ca="1">X22*$V$44</f>
         <v>0</v>
       </c>
       <c r="Z22" s="4">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="7"/>
         <v>0</v>
       </c>
       <c r="AA22" s="4">
@@ -2506,186 +2557,200 @@
         <v>0.85000000000000009</v>
       </c>
     </row>
-    <row r="23" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B23" s="78"/>
+    <row r="23" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B23" s="90"/>
       <c r="C23" s="58">
         <v>5</v>
       </c>
       <c r="D23" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="E23" s="65"/>
-      <c r="F23" s="66"/>
+      <c r="E23" s="65">
+        <v>2177448</v>
+      </c>
+      <c r="F23" s="66" t="s">
+        <v>100</v>
+      </c>
       <c r="G23" s="30">
-        <v>0.15</v>
+        <f t="shared" si="2"/>
+        <v>0.16666666666666669</v>
       </c>
       <c r="H23" s="8">
-        <v>0.15</v>
+        <f t="shared" si="2"/>
+        <v>0.16666666666666669</v>
       </c>
       <c r="I23" s="31">
-        <v>0.15</v>
-      </c>
-      <c r="J23" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="2"/>
+        <v>0.16666666666666669</v>
+      </c>
+      <c r="J23" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K23" s="100">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.71399999999999997</v>
+      <c r="K23" s="78">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.85000000000000009</v>
       </c>
       <c r="L23" s="34"/>
       <c r="M23" s="46">
-        <f>E23</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>2177448</v>
       </c>
       <c r="N23" s="68">
         <f t="array" ref="N23">SUM(G23:I23/$G$17:$I$17*$G$16:$I$16)</f>
-        <v>0.15</v>
+        <v>0.16666666666666669</v>
       </c>
       <c r="O23" s="68">
-        <f t="shared" ref="O23:O43" si="5">1/$M$49</f>
-        <v>0.25</v>
+        <f t="shared" ref="O23:O43" si="8">1/$M$49</f>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P23" s="4">
-        <f t="shared" ref="P23:P43" si="6">N23/O23</f>
-        <v>0.6</v>
+        <f t="shared" ref="P23:P43" si="9">N23/O23</f>
+        <v>1.0000000000000002</v>
       </c>
       <c r="Q23" s="4">
-        <f t="shared" ref="Q23:Q43" si="7">$G$5</f>
+        <f t="shared" ref="Q23:Q43" si="10">$G$5</f>
         <v>0.85</v>
       </c>
       <c r="R23" s="4">
-        <f t="shared" ref="R23:R43" si="8">Q23*$G$7</f>
+        <f t="shared" ref="R23:R43" si="11">Q23*$G$7</f>
         <v>0.51</v>
       </c>
       <c r="S23" s="4">
-        <f t="shared" ref="S23:S43" si="9">P23*Q23*$G$8</f>
-        <v>0.20400000000000001</v>
+        <f t="shared" ref="S23:S43" si="12">P23*Q23*$G$8</f>
+        <v>0.34000000000000008</v>
       </c>
       <c r="T23" s="4">
-        <f t="shared" ref="T23:T43" si="10">SUM(R23:S23)</f>
-        <v>0.71399999999999997</v>
+        <f t="shared" ref="T23:T43" si="13">SUM(R23:S23)</f>
+        <v>0.85000000000000009</v>
       </c>
       <c r="U23" s="4">
-        <f t="shared" ref="U23:U43" si="11">MIN(1,T23)</f>
-        <v>0.71399999999999997</v>
+        <f t="shared" ref="U23:U43" si="14">MIN(1,T23)</f>
+        <v>0.85000000000000009</v>
       </c>
       <c r="V23" s="4">
-        <f t="shared" ref="V23:V43" si="12">T23-U23</f>
+        <f t="shared" ref="V23:V43" si="15">T23-U23</f>
         <v>0</v>
       </c>
       <c r="W23" s="4">
-        <f t="shared" ref="W23:W43" si="13">1-U23</f>
-        <v>0.28600000000000003</v>
+        <f t="shared" ref="W23:W43" si="16">1-U23</f>
+        <v>0.14999999999999991</v>
       </c>
       <c r="X23" s="4">
-        <f t="shared" ref="X23:X43" ca="1" si="14">W23/$W$44</f>
-        <v>0.47666666666666702</v>
+        <f t="shared" ref="X23:X43" ca="1" si="17">W23/$W$44</f>
+        <v>0.16666666666666666</v>
       </c>
       <c r="Y23" s="4">
-        <f t="shared" ref="Y23:Y43" ca="1" si="15">X23*$V$44</f>
+        <f t="shared" ref="Y23:Y43" ca="1" si="18">X23*$V$44</f>
         <v>0</v>
       </c>
       <c r="Z23" s="4">
-        <f t="shared" ref="Z23:Z43" ca="1" si="16">Y23*$G$10</f>
+        <f t="shared" ref="Z23:Z43" ca="1" si="19">Y23*$G$10</f>
         <v>0</v>
       </c>
       <c r="AA23" s="4">
-        <f t="shared" ref="AA23:AA43" ca="1" si="17">U23+Z23</f>
-        <v>0.71399999999999997</v>
-      </c>
-    </row>
-    <row r="24" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B24" s="78"/>
+        <f t="shared" ref="AA23:AA43" ca="1" si="20">U23+Z23</f>
+        <v>0.85000000000000009</v>
+      </c>
+    </row>
+    <row r="24" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B24" s="90"/>
       <c r="C24" s="58">
         <v>6</v>
       </c>
       <c r="D24" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="E24" s="65"/>
-      <c r="F24" s="66"/>
+      <c r="E24" s="65">
+        <v>2363434</v>
+      </c>
+      <c r="F24" s="66" t="s">
+        <v>101</v>
+      </c>
       <c r="G24" s="30">
-        <v>0.35</v>
+        <f t="shared" si="2"/>
+        <v>0.16666666666666669</v>
       </c>
       <c r="H24" s="8">
-        <v>0.35</v>
+        <f t="shared" si="2"/>
+        <v>0.16666666666666669</v>
       </c>
       <c r="I24" s="31">
-        <v>0.25</v>
-      </c>
-      <c r="J24" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="2"/>
+        <v>0.16666666666666669</v>
+      </c>
+      <c r="J24" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K24" s="100">
-        <f t="shared" ca="1" si="1"/>
-        <v>0.95879999999999999</v>
+      <c r="K24" s="78">
+        <f t="shared" ca="1" si="4"/>
+        <v>0.85000000000000009</v>
       </c>
       <c r="L24" s="34"/>
       <c r="M24" s="46">
-        <f>E24</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>2363434</v>
       </c>
       <c r="N24" s="68">
         <f t="array" ref="N24">SUM(G24:I24/$G$17:$I$17*$G$16:$I$16)</f>
-        <v>0.32999999999999996</v>
+        <v>0.16666666666666669</v>
       </c>
       <c r="O24" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P24" s="4">
-        <f t="shared" si="6"/>
-        <v>1.3199999999999998</v>
+        <f t="shared" si="9"/>
+        <v>1.0000000000000002</v>
       </c>
       <c r="Q24" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R24" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S24" s="4">
-        <f t="shared" si="9"/>
-        <v>0.44879999999999998</v>
+        <f t="shared" si="12"/>
+        <v>0.34000000000000008</v>
       </c>
       <c r="T24" s="4">
-        <f t="shared" si="10"/>
-        <v>0.95879999999999999</v>
+        <f t="shared" si="13"/>
+        <v>0.85000000000000009</v>
       </c>
       <c r="U24" s="4">
-        <f t="shared" si="11"/>
-        <v>0.95879999999999999</v>
+        <f t="shared" si="14"/>
+        <v>0.85000000000000009</v>
       </c>
       <c r="V24" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W24" s="4">
-        <f t="shared" si="13"/>
-        <v>4.1200000000000014E-2</v>
+        <f t="shared" si="16"/>
+        <v>0.14999999999999991</v>
       </c>
       <c r="X24" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>6.8666666666666737E-2</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="Y24" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z24" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA24" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.95879999999999999</v>
-      </c>
-    </row>
-    <row r="25" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B25" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.85000000000000009</v>
+      </c>
+    </row>
+    <row r="25" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B25" s="90"/>
       <c r="C25" s="58">
         <v>7</v>
       </c>
@@ -2697,17 +2762,17 @@
       <c r="G25" s="30"/>
       <c r="H25" s="8"/>
       <c r="I25" s="31"/>
-      <c r="J25" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J25" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K25" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K25" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L25" s="34"/>
       <c r="M25" s="46">
-        <f>E25</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N25" s="68">
@@ -2715,60 +2780,60 @@
         <v>0</v>
       </c>
       <c r="O25" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P25" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q25" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R25" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S25" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T25" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U25" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V25" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W25" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X25" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y25" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z25" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA25" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="26" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B26" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="26" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B26" s="90"/>
       <c r="C26" s="58">
         <v>8</v>
       </c>
@@ -2780,17 +2845,17 @@
       <c r="G26" s="30"/>
       <c r="H26" s="8"/>
       <c r="I26" s="31"/>
-      <c r="J26" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J26" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K26" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K26" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L26" s="34"/>
       <c r="M26" s="46">
-        <f>E26</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N26" s="68">
@@ -2798,60 +2863,60 @@
         <v>0</v>
       </c>
       <c r="O26" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P26" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q26" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R26" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S26" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T26" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U26" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V26" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W26" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X26" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y26" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z26" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA26" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="27" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B27" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="27" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B27" s="90"/>
       <c r="C27" s="58">
         <v>9</v>
       </c>
@@ -2863,17 +2928,17 @@
       <c r="G27" s="30"/>
       <c r="H27" s="8"/>
       <c r="I27" s="31"/>
-      <c r="J27" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J27" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K27" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K27" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L27" s="34"/>
       <c r="M27" s="46">
-        <f>E27</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N27" s="68">
@@ -2881,60 +2946,60 @@
         <v>0</v>
       </c>
       <c r="O27" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P27" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q27" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R27" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S27" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T27" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U27" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V27" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W27" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X27" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y27" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z27" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA27" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="28" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B28" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="28" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B28" s="90"/>
       <c r="C28" s="58">
         <v>10</v>
       </c>
@@ -2946,17 +3011,17 @@
       <c r="G28" s="30"/>
       <c r="H28" s="8"/>
       <c r="I28" s="31"/>
-      <c r="J28" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J28" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K28" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K28" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L28" s="34"/>
       <c r="M28" s="46">
-        <f>E28</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N28" s="68">
@@ -2964,60 +3029,60 @@
         <v>0</v>
       </c>
       <c r="O28" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P28" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q28" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R28" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S28" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T28" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U28" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V28" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W28" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X28" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y28" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z28" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA28" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="29" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B29" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="29" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B29" s="90"/>
       <c r="C29" s="58">
         <v>11</v>
       </c>
@@ -3029,17 +3094,17 @@
       <c r="G29" s="30"/>
       <c r="H29" s="8"/>
       <c r="I29" s="31"/>
-      <c r="J29" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J29" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K29" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K29" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L29" s="34"/>
       <c r="M29" s="46">
-        <f>E29</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N29" s="68">
@@ -3047,60 +3112,60 @@
         <v>0</v>
       </c>
       <c r="O29" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P29" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q29" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R29" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S29" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T29" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U29" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V29" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W29" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X29" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y29" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z29" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA29" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="30" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B30" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="30" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B30" s="90"/>
       <c r="C30" s="58">
         <v>12</v>
       </c>
@@ -3112,17 +3177,17 @@
       <c r="G30" s="30"/>
       <c r="H30" s="8"/>
       <c r="I30" s="31"/>
-      <c r="J30" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J30" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K30" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K30" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L30" s="34"/>
       <c r="M30" s="46">
-        <f>E30</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N30" s="68">
@@ -3130,60 +3195,60 @@
         <v>0</v>
       </c>
       <c r="O30" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P30" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q30" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R30" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S30" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T30" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U30" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V30" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W30" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X30" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y30" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z30" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA30" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="31" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B31" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="31" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B31" s="90"/>
       <c r="C31" s="58">
         <v>13</v>
       </c>
@@ -3195,17 +3260,17 @@
       <c r="G31" s="30"/>
       <c r="H31" s="8"/>
       <c r="I31" s="31"/>
-      <c r="J31" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J31" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K31" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K31" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L31" s="34"/>
       <c r="M31" s="46">
-        <f>E31</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N31" s="68">
@@ -3213,60 +3278,60 @@
         <v>0</v>
       </c>
       <c r="O31" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P31" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q31" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R31" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S31" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T31" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U31" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V31" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W31" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X31" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y31" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z31" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA31" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="32" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B32" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="32" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B32" s="90"/>
       <c r="C32" s="58">
         <v>14</v>
       </c>
@@ -3278,17 +3343,17 @@
       <c r="G32" s="30"/>
       <c r="H32" s="8"/>
       <c r="I32" s="31"/>
-      <c r="J32" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J32" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K32" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K32" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L32" s="34"/>
       <c r="M32" s="46">
-        <f>E32</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N32" s="68">
@@ -3296,60 +3361,60 @@
         <v>0</v>
       </c>
       <c r="O32" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P32" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q32" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R32" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S32" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T32" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U32" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V32" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W32" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X32" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y32" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z32" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA32" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="33" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B33" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="33" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B33" s="90"/>
       <c r="C33" s="58">
         <v>15</v>
       </c>
@@ -3361,17 +3426,17 @@
       <c r="G33" s="30"/>
       <c r="H33" s="8"/>
       <c r="I33" s="31"/>
-      <c r="J33" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J33" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K33" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K33" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L33" s="34"/>
       <c r="M33" s="46">
-        <f>E33</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N33" s="68">
@@ -3379,60 +3444,60 @@
         <v>0</v>
       </c>
       <c r="O33" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P33" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q33" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R33" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S33" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T33" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U33" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V33" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W33" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X33" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y33" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z33" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA33" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="34" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B34" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="34" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B34" s="90"/>
       <c r="C34" s="58">
         <v>16</v>
       </c>
@@ -3444,17 +3509,17 @@
       <c r="G34" s="30"/>
       <c r="H34" s="8"/>
       <c r="I34" s="31"/>
-      <c r="J34" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J34" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K34" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K34" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L34" s="34"/>
       <c r="M34" s="46">
-        <f>E34</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N34" s="68">
@@ -3462,60 +3527,60 @@
         <v>0</v>
       </c>
       <c r="O34" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P34" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q34" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R34" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S34" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T34" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U34" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V34" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W34" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X34" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y34" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z34" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA34" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="35" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B35" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="35" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B35" s="90"/>
       <c r="C35" s="58">
         <v>17</v>
       </c>
@@ -3527,17 +3592,17 @@
       <c r="G35" s="30"/>
       <c r="H35" s="8"/>
       <c r="I35" s="31"/>
-      <c r="J35" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J35" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K35" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K35" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L35" s="34"/>
       <c r="M35" s="46">
-        <f>E35</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N35" s="68">
@@ -3545,60 +3610,60 @@
         <v>0</v>
       </c>
       <c r="O35" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P35" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q35" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R35" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S35" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T35" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U35" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V35" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W35" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X35" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y35" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z35" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA35" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="36" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B36" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="36" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B36" s="90"/>
       <c r="C36" s="58">
         <v>18</v>
       </c>
@@ -3610,17 +3675,17 @@
       <c r="G36" s="30"/>
       <c r="H36" s="8"/>
       <c r="I36" s="31"/>
-      <c r="J36" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J36" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K36" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K36" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L36" s="34"/>
       <c r="M36" s="46">
-        <f>E36</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N36" s="68">
@@ -3628,60 +3693,60 @@
         <v>0</v>
       </c>
       <c r="O36" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P36" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q36" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R36" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S36" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T36" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U36" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V36" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W36" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X36" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y36" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z36" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA36" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="37" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B37" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="37" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="90"/>
       <c r="C37" s="58">
         <v>19</v>
       </c>
@@ -3693,17 +3758,17 @@
       <c r="G37" s="30"/>
       <c r="H37" s="8"/>
       <c r="I37" s="31"/>
-      <c r="J37" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J37" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K37" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K37" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L37" s="34"/>
       <c r="M37" s="46">
-        <f>E37</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N37" s="68">
@@ -3711,60 +3776,60 @@
         <v>0</v>
       </c>
       <c r="O37" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P37" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q37" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R37" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S37" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T37" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U37" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V37" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W37" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X37" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y37" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z37" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA37" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="38" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B38" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="38" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B38" s="90"/>
       <c r="C38" s="58">
         <v>20</v>
       </c>
@@ -3776,17 +3841,17 @@
       <c r="G38" s="30"/>
       <c r="H38" s="8"/>
       <c r="I38" s="31"/>
-      <c r="J38" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J38" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K38" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K38" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L38" s="34"/>
       <c r="M38" s="46">
-        <f>E38</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N38" s="68">
@@ -3794,60 +3859,60 @@
         <v>0</v>
       </c>
       <c r="O38" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P38" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q38" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R38" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S38" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T38" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U38" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V38" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W38" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X38" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y38" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z38" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA38" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="39" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B39" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="39" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B39" s="90"/>
       <c r="C39" s="58">
         <v>21</v>
       </c>
@@ -3859,17 +3924,17 @@
       <c r="G39" s="30"/>
       <c r="H39" s="8"/>
       <c r="I39" s="31"/>
-      <c r="J39" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J39" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K39" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K39" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L39" s="34"/>
       <c r="M39" s="46">
-        <f>E39</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N39" s="68">
@@ -3877,60 +3942,60 @@
         <v>0</v>
       </c>
       <c r="O39" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P39" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q39" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R39" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S39" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T39" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U39" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V39" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W39" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X39" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y39" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z39" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA39" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="40" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B40" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="40" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B40" s="90"/>
       <c r="C40" s="58">
         <v>22</v>
       </c>
@@ -3942,17 +4007,17 @@
       <c r="G40" s="30"/>
       <c r="H40" s="8"/>
       <c r="I40" s="31"/>
-      <c r="J40" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J40" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K40" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K40" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L40" s="34"/>
       <c r="M40" s="46">
-        <f>E40</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N40" s="68">
@@ -3960,60 +4025,60 @@
         <v>0</v>
       </c>
       <c r="O40" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P40" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q40" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R40" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S40" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T40" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U40" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V40" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W40" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X40" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y40" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z40" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA40" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="41" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B41" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="41" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B41" s="90"/>
       <c r="C41" s="58">
         <v>23</v>
       </c>
@@ -4025,17 +4090,17 @@
       <c r="G41" s="30"/>
       <c r="H41" s="8"/>
       <c r="I41" s="31"/>
-      <c r="J41" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J41" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K41" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K41" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L41" s="34"/>
       <c r="M41" s="46">
-        <f>E41</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N41" s="68">
@@ -4043,60 +4108,60 @@
         <v>0</v>
       </c>
       <c r="O41" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P41" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q41" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R41" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S41" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T41" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U41" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V41" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W41" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X41" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y41" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z41" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA41" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="42" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B42" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="42" spans="2:27" s="67" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B42" s="90"/>
       <c r="C42" s="58">
         <v>24</v>
       </c>
@@ -4108,17 +4173,17 @@
       <c r="G42" s="30"/>
       <c r="H42" s="8"/>
       <c r="I42" s="31"/>
-      <c r="J42" s="99" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="J42" s="77" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K42" s="100">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K42" s="78">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L42" s="34"/>
       <c r="M42" s="46">
-        <f>E42</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N42" s="68">
@@ -4126,82 +4191,82 @@
         <v>0</v>
       </c>
       <c r="O42" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P42" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q42" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R42" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S42" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T42" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U42" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V42" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W42" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X42" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y42" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z42" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA42" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="43" spans="2:27" s="67" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B43" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="43" spans="2:27" s="67" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B43" s="90"/>
       <c r="C43" s="58">
         <v>25</v>
       </c>
-      <c r="D43" s="91" t="s">
+      <c r="D43" s="69" t="s">
         <v>74</v>
       </c>
-      <c r="E43" s="92"/>
-      <c r="F43" s="93"/>
-      <c r="G43" s="94"/>
-      <c r="H43" s="95"/>
-      <c r="I43" s="96"/>
-      <c r="J43" s="97" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="E43" s="70"/>
+      <c r="F43" s="71"/>
+      <c r="G43" s="72"/>
+      <c r="H43" s="73"/>
+      <c r="I43" s="74"/>
+      <c r="J43" s="75" t="str">
+        <f t="shared" ca="1" si="3"/>
         <v/>
       </c>
-      <c r="K43" s="98">
-        <f t="shared" ca="1" si="1"/>
+      <c r="K43" s="76">
+        <f t="shared" ca="1" si="4"/>
         <v>0.51</v>
       </c>
       <c r="L43" s="34"/>
       <c r="M43" s="46">
-        <f>E43</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N43" s="68">
@@ -4209,79 +4274,79 @@
         <v>0</v>
       </c>
       <c r="O43" s="68">
-        <f t="shared" si="5"/>
-        <v>0.25</v>
+        <f t="shared" si="8"/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="P43" s="4">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Q43" s="4">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>0.85</v>
       </c>
       <c r="R43" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.51</v>
       </c>
       <c r="S43" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T43" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.51</v>
       </c>
       <c r="U43" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.51</v>
       </c>
       <c r="V43" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="W43" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>0.49</v>
       </c>
       <c r="X43" s="4">
-        <f t="shared" ca="1" si="14"/>
-        <v>0.8166666666666671</v>
+        <f t="shared" ca="1" si="17"/>
+        <v>0.54444444444444473</v>
       </c>
       <c r="Y43" s="4">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="18"/>
         <v>0</v>
       </c>
       <c r="Z43" s="4">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="19"/>
         <v>0</v>
       </c>
       <c r="AA43" s="4">
-        <f t="shared" ca="1" si="17"/>
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="44" spans="2:27" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B44" s="78"/>
+        <f t="shared" ca="1" si="20"/>
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="44" spans="2:27" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B44" s="90"/>
       <c r="D44" s="19"/>
       <c r="E44" s="10"/>
       <c r="F44" s="10"/>
       <c r="G44" s="32">
         <f ca="1">SUM(OFFSET(G19, 0, 0, $G$3, 1))</f>
-        <v>1</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="H44" s="11">
-        <f t="shared" ref="H44:I44" ca="1" si="18">SUM(OFFSET(H19, 0, 0, $G$3, 1))</f>
-        <v>1</v>
+        <f t="shared" ref="H44:I44" ca="1" si="21">SUM(OFFSET(H19, 0, 0, $G$3, 1))</f>
+        <v>1.0000000000000002</v>
       </c>
       <c r="I44" s="33">
-        <f t="shared" ca="1" si="18"/>
-        <v>1</v>
+        <f t="shared" ca="1" si="21"/>
+        <v>1.0000000000000002</v>
       </c>
       <c r="J44" s="11"/>
       <c r="K44" s="20">
         <f ca="1">AVERAGE(OFFSET(K19, 0, 0, $G$3, 1))</f>
-        <v>0.85000000000000009</v>
+        <v>0.85</v>
       </c>
       <c r="L44" s="34"/>
       <c r="M44" s="5" t="s">
@@ -4289,11 +4354,11 @@
       </c>
       <c r="N44" s="4">
         <f>SUM(N19:N22)</f>
-        <v>1</v>
+        <v>0.66666666666666674</v>
       </c>
       <c r="O44" s="4">
         <f>SUM(O19:O22)</f>
-        <v>1</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="P44" s="4"/>
       <c r="Q44" s="4"/>
@@ -4307,13 +4372,13 @@
       </c>
       <c r="W44" s="4">
         <f ca="1">SUM(OFFSET(W19, 0, 0, $G$3, 1))</f>
-        <v>0.59999999999999964</v>
+        <v>0.89999999999999947</v>
       </c>
       <c r="X44" s="2"/>
       <c r="Y44" s="2"/>
     </row>
-    <row r="45" spans="2:27" s="6" customFormat="1" ht="14.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="B45" s="78"/>
+    <row r="45" spans="2:27" s="6" customFormat="1" ht="14.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B45" s="90"/>
       <c r="G45" s="54"/>
       <c r="H45" s="37"/>
       <c r="I45" s="37"/>
@@ -4327,18 +4392,18 @@
       <c r="O45" s="2"/>
       <c r="P45" s="4">
         <f>AVERAGE(P19:P22)</f>
-        <v>1</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="Q45" s="4">
         <f>AVERAGE(Q19:Q22)</f>
         <v>0.85</v>
       </c>
       <c r="R45" s="4">
-        <f t="shared" ref="R45:S45" si="19">AVERAGE(R19:R22)</f>
+        <f t="shared" ref="R45:S45" si="22">AVERAGE(R19:R22)</f>
         <v>0.51</v>
       </c>
       <c r="S45" s="4">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>0.34000000000000008</v>
       </c>
       <c r="T45" s="4">
@@ -4356,7 +4421,7 @@
       <c r="Z45" s="2"/>
       <c r="AA45" s="2"/>
     </row>
-    <row r="46" spans="2:27" s="6" customFormat="1" ht="12.4" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="2:27" s="6" customFormat="1" ht="12.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B46" s="55"/>
       <c r="G46" s="57" t="s">
         <v>52</v>
@@ -4386,17 +4451,17 @@
       <c r="Z46" s="2"/>
       <c r="AA46" s="2"/>
     </row>
-    <row r="47" spans="2:27" s="6" customFormat="1" ht="31.15" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="2:27" s="6" customFormat="1" ht="31.15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="G47" s="56" t="str">
         <f ca="1">IF(G44&lt;&gt;1,"La somme doit être égale à 100%","")</f>
         <v/>
       </c>
       <c r="H47" s="56" t="str">
-        <f t="shared" ref="H47:I47" ca="1" si="20">IF(H44&lt;&gt;1,"La somme doit être égale à 100%","")</f>
+        <f t="shared" ref="H47:I47" ca="1" si="23">IF(H44&lt;&gt;1,"La somme doit être égale à 100%","")</f>
         <v/>
       </c>
       <c r="I47" s="56" t="str">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="23"/>
         <v/>
       </c>
       <c r="J47" s="56"/>
@@ -4418,7 +4483,7 @@
       <c r="Z47" s="2"/>
       <c r="AA47" s="2"/>
     </row>
-    <row r="48" spans="2:27" s="6" customFormat="1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="48" spans="2:27" s="6" customFormat="1" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="H48" s="37"/>
       <c r="I48" s="37"/>
       <c r="J48" s="37"/>
@@ -4470,7 +4535,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="49" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="49" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E49" s="43"/>
       <c r="F49" s="43"/>
       <c r="G49" s="40"/>
@@ -4483,7 +4548,7 @@
       <c r="L49" s="38"/>
       <c r="M49" s="59">
         <f>G3</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N49" s="41"/>
       <c r="O49" s="41"/>
@@ -4500,7 +4565,7 @@
       <c r="Z49" s="41"/>
       <c r="AA49" s="41"/>
     </row>
-    <row r="50" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="50" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E50" s="48"/>
       <c r="F50" s="43"/>
       <c r="G50" s="40"/>
@@ -4527,7 +4592,7 @@
       <c r="Z50" s="41"/>
       <c r="AA50" s="41"/>
     </row>
-    <row r="51" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="51" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E51" s="48"/>
       <c r="F51" s="43"/>
       <c r="G51" s="40"/>
@@ -4554,7 +4619,7 @@
       <c r="Z51" s="41"/>
       <c r="AA51" s="41"/>
     </row>
-    <row r="52" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="52" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E52" s="48"/>
       <c r="F52" s="43"/>
       <c r="G52" s="40"/>
@@ -4581,7 +4646,7 @@
       <c r="Z52" s="41"/>
       <c r="AA52" s="41"/>
     </row>
-    <row r="53" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E53" s="48"/>
       <c r="F53" s="43"/>
       <c r="G53" s="40"/>
@@ -4608,7 +4673,7 @@
       <c r="Z53" s="41"/>
       <c r="AA53" s="41"/>
     </row>
-    <row r="54" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="54" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E54" s="48"/>
       <c r="F54" s="43"/>
       <c r="G54" s="40"/>
@@ -4635,7 +4700,7 @@
       <c r="Z54" s="41"/>
       <c r="AA54" s="41"/>
     </row>
-    <row r="55" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="55" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E55" s="48"/>
       <c r="F55" s="43"/>
       <c r="G55" s="40"/>
@@ -4662,7 +4727,7 @@
       <c r="Z55" s="41"/>
       <c r="AA55" s="41"/>
     </row>
-    <row r="56" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="56" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E56" s="48"/>
       <c r="F56" s="43"/>
       <c r="G56" s="40"/>
@@ -4689,7 +4754,7 @@
       <c r="Z56" s="41"/>
       <c r="AA56" s="41"/>
     </row>
-    <row r="57" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="57" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E57" s="48"/>
       <c r="F57" s="43"/>
       <c r="G57" s="40"/>
@@ -4716,7 +4781,7 @@
       <c r="Z57" s="41"/>
       <c r="AA57" s="41"/>
     </row>
-    <row r="58" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="58" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E58" s="48"/>
       <c r="F58" s="43"/>
       <c r="G58" s="40"/>
@@ -4743,7 +4808,7 @@
       <c r="Z58" s="41"/>
       <c r="AA58" s="41"/>
     </row>
-    <row r="59" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="59" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E59" s="48"/>
       <c r="F59" s="43"/>
       <c r="G59" s="40"/>
@@ -4770,7 +4835,7 @@
       <c r="Z59" s="41"/>
       <c r="AA59" s="41"/>
     </row>
-    <row r="60" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="60" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E60" s="48"/>
       <c r="F60" s="43"/>
       <c r="G60" s="40"/>
@@ -4797,7 +4862,7 @@
       <c r="Z60" s="41"/>
       <c r="AA60" s="41"/>
     </row>
-    <row r="61" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="61" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E61" s="48"/>
       <c r="F61" s="43"/>
       <c r="G61" s="40"/>
@@ -4824,7 +4889,7 @@
       <c r="Z61" s="41"/>
       <c r="AA61" s="41"/>
     </row>
-    <row r="62" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="62" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E62" s="48"/>
       <c r="F62" s="43"/>
       <c r="G62" s="40"/>
@@ -4851,7 +4916,7 @@
       <c r="Z62" s="42"/>
       <c r="AA62" s="41"/>
     </row>
-    <row r="63" spans="5:27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="63" spans="5:27" hidden="1" x14ac:dyDescent="0.35">
       <c r="E63" s="48"/>
       <c r="F63" s="43"/>
       <c r="G63" s="40"/>
@@ -4878,86 +4943,88 @@
       <c r="Z63" s="40"/>
       <c r="AA63" s="42"/>
     </row>
-    <row r="64" spans="5:27" hidden="1" x14ac:dyDescent="0.45"/>
-    <row r="65" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="64" spans="5:27" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="65" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L65" s="38" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="66" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="66" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L66" s="38" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="67" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="67" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L67" s="38" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="68" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="68" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L68" s="38" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="69" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="69" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L69" s="38" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="70" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L70" s="38" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="71" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="71" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L71" s="38" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="72" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L72" s="38" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="73" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="73" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L73" s="38" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="74" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="74" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L74" s="38" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="75" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="75" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L75" s="38" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="76" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="76" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L76" s="38" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="77" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="77" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L77" s="38" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="78" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="78" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L78" s="38" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="79" spans="12:12" hidden="1" x14ac:dyDescent="0.45">
+    <row r="79" spans="12:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="L79" s="38" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="80" spans="12:12" hidden="1" x14ac:dyDescent="0.45"/>
+    <row r="80" spans="12:12" hidden="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="d2wj9CCEuGw4Mg6otQpiYDLe9ScqX7RqQ3VxEP8wAjD/h08OAkcxvAV0OuVlGLs0lDzKZe11zE9KnrJqQ3HHBQ==" saltValue="cDUUGHebzs7qC23bO1RmFA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="17">
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="G11:K11"/>
     <mergeCell ref="B2:B12"/>
     <mergeCell ref="B14:B45"/>
     <mergeCell ref="G10:K10"/>
@@ -4973,12 +5040,10 @@
     <mergeCell ref="D5:F5"/>
     <mergeCell ref="D3:F3"/>
     <mergeCell ref="G3:K3"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="G11:K11"/>
   </mergeCells>
-  <conditionalFormatting sqref="G16:J16">
-    <cfRule type="expression" dxfId="3" priority="4">
-      <formula>SUM($G$16:$I$16)&lt;&gt;1</formula>
+  <conditionalFormatting sqref="D19:K43">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>$C19&gt;$G$3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G19:I44">
@@ -4986,14 +5051,14 @@
       <formula>LEN(G$47)&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G46:J46">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>LEN(G47)&lt;&gt;0</formula>
+  <conditionalFormatting sqref="G16:J16">
+    <cfRule type="expression" dxfId="1" priority="4">
+      <formula>SUM($G$16:$I$16)&lt;&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D19:K43">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>$C19&gt;$G$3</formula>
+  <conditionalFormatting sqref="G46:J46">
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>LEN(G47)&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations xWindow="1991" yWindow="1205" count="13">
@@ -5048,127 +5113,127 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E086803D-69FD-4B55-9FDE-B06A5092F69F}">
   <dimension ref="B2:E29"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.59765625" style="67" customWidth="1"/>
-    <col min="2" max="2" width="9.06640625" style="67" customWidth="1"/>
-    <col min="3" max="3" width="12.6640625" style="67" customWidth="1"/>
-    <col min="4" max="4" width="93.53125" style="67" customWidth="1"/>
+    <col min="1" max="1" width="2.6328125" style="67" customWidth="1"/>
+    <col min="2" max="2" width="9.08984375" style="67" customWidth="1"/>
+    <col min="3" max="3" width="12.6328125" style="67" customWidth="1"/>
+    <col min="4" max="4" width="93.54296875" style="67" customWidth="1"/>
     <col min="5" max="5" width="2" style="67" customWidth="1"/>
-    <col min="6" max="16384" width="9.06640625" style="67"/>
+    <col min="6" max="16384" width="9.08984375" style="67"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" s="67" customFormat="1" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B2" s="113" t="s">
+    <row r="2" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B2" s="83" t="s">
         <v>93</v>
       </c>
-      <c r="C2" s="113"/>
-      <c r="D2" s="113"/>
-      <c r="E2" s="113"/>
-    </row>
-    <row r="3" spans="2:5" s="67" customFormat="1" ht="5.75" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="4" spans="2:5" s="67" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="C2" s="83"/>
+      <c r="D2" s="83"/>
+      <c r="E2" s="83"/>
+    </row>
+    <row r="3" spans="2:5" ht="5.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B4" s="67" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="2:5" s="67" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="67" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="8" spans="2:5" s="67" customFormat="1" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B8" s="113" t="s">
+    <row r="8" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B8" s="83" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="113"/>
-      <c r="D8" s="113"/>
-      <c r="E8" s="113"/>
-    </row>
-    <row r="9" spans="2:5" s="67" customFormat="1" ht="5.75" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="10" spans="2:5" s="67" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="C8" s="83"/>
+      <c r="D8" s="83"/>
+      <c r="E8" s="83"/>
+    </row>
+    <row r="9" spans="2:5" ht="5.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="67" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="2:5" s="67" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="67">
         <v>1</v>
       </c>
-      <c r="C11" s="114" t="s">
+      <c r="C11" s="84" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="67" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="12" spans="2:5" s="67" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="C12" s="114"/>
-      <c r="D12" s="115" t="s">
+    <row r="12" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="C12" s="84"/>
+      <c r="D12" s="85" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="13" spans="2:5" s="67" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="67">
         <v>2</v>
       </c>
-      <c r="C13" s="114" t="s">
+      <c r="C13" s="84" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="67" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="2:5" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="C14" s="114"/>
-      <c r="D14" s="116" t="s">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="C14" s="84"/>
+      <c r="D14" s="86" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="15" spans="2:5" s="67" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="67">
         <v>3</v>
       </c>
-      <c r="C15" s="114" t="s">
+      <c r="C15" s="84" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="67" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="16" spans="2:5" s="67" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="D16" s="116" t="s">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="D16" s="86" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="18" spans="2:5" s="67" customFormat="1" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B18" s="113" t="s">
+    <row r="18" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B18" s="83" t="s">
         <v>85</v>
       </c>
-      <c r="C18" s="113"/>
-      <c r="D18" s="113"/>
-      <c r="E18" s="113"/>
-    </row>
-    <row r="19" spans="2:5" s="67" customFormat="1" ht="5.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="20" spans="2:5" s="67" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="C20" s="111" t="s">
+      <c r="C18" s="83"/>
+      <c r="D18" s="83"/>
+      <c r="E18" s="83"/>
+    </row>
+    <row r="19" spans="2:5" ht="5.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="20" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C20" s="116" t="s">
         <v>86</v>
       </c>
-      <c r="D20" s="112"/>
-    </row>
-    <row r="21" spans="2:5" s="67" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="C21" s="117" t="s">
+      <c r="D20" s="117"/>
+    </row>
+    <row r="21" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C21" s="115" t="s">
         <v>87</v>
       </c>
-      <c r="D21" s="117"/>
-    </row>
-    <row r="22" spans="2:5" s="67" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="D21" s="115"/>
+    </row>
+    <row r="22" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C22" s="118" t="s">
         <v>88</v>
       </c>
       <c r="D22" s="118"/>
     </row>
-    <row r="24" spans="2:5" s="67" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B24" s="67">
         <v>1</v>
       </c>
@@ -5176,7 +5241,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="25" spans="2:5" s="67" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B25" s="67">
         <v>2</v>
       </c>
@@ -5184,7 +5249,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="26" spans="2:5" s="67" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B26" s="67">
         <v>3</v>
       </c>
@@ -5192,12 +5257,12 @@
         <v>90</v>
       </c>
     </row>
-    <row r="27" spans="2:5" s="67" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
       <c r="C27" s="67" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="29" spans="2:5" s="67" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B29" s="119" t="s">
         <v>92</v>
       </c>

</xml_diff>